<commit_message>
chore: sync pipeline September state
</commit_message>
<xml_diff>
--- a/2_planilla/inputs/lecturas/lecturas_planilla_2026-08.xlsx
+++ b/2_planilla/inputs/lecturas/lecturas_planilla_2026-08.xlsx
@@ -708,7 +708,7 @@
         </is>
       </c>
       <c r="I3" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="I4" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="I5" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="I6" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
@@ -872,7 +872,7 @@
         </is>
       </c>
       <c r="I7" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="I8" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="I9" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="I10" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="I11" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="I12" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="I13" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -1161,7 +1161,7 @@
         </is>
       </c>
       <c r="I14" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="I15" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="I16" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="I17" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="I18" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1366,7 +1366,7 @@
         </is>
       </c>
       <c r="I19" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="I20" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="I21" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="I22" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="I23" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="I24" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="I25" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="I26" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="I27" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="I28" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
@@ -1776,7 +1776,7 @@
         </is>
       </c>
       <c r="I29" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="I30" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="I31" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="I32" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="I33" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="I34" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2022,7 +2022,7 @@
         </is>
       </c>
       <c r="I35" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="I36" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="I37" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="I38" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2186,7 +2186,7 @@
         </is>
       </c>
       <c r="I39" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -2227,7 +2227,7 @@
         </is>
       </c>
       <c r="I40" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -2268,7 +2268,7 @@
         </is>
       </c>
       <c r="I41" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="I42" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="I43" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="I44" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="I45" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="I46" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
@@ -2514,7 +2514,7 @@
         </is>
       </c>
       <c r="I47" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="I48" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
@@ -2596,7 +2596,7 @@
         </is>
       </c>
       <c r="I49" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="I50" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="I51" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="I52" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="I53" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="I54" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
@@ -2842,7 +2842,7 @@
         </is>
       </c>
       <c r="I55" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="I56" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
@@ -2924,7 +2924,7 @@
         </is>
       </c>
       <c r="I57" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="I58" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
@@ -3006,7 +3006,7 @@
         </is>
       </c>
       <c r="I59" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="I60" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
@@ -3088,7 +3088,7 @@
         </is>
       </c>
       <c r="I61" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="I62" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
@@ -3170,7 +3170,7 @@
         </is>
       </c>
       <c r="I63" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="I64" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1">
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="I65" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="I66" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
@@ -3334,7 +3334,7 @@
         </is>
       </c>
       <c r="I67" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
@@ -3375,7 +3375,7 @@
         </is>
       </c>
       <c r="I68" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="I69" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="I70" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
@@ -3498,7 +3498,7 @@
         </is>
       </c>
       <c r="I71" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
@@ -3539,7 +3539,7 @@
         </is>
       </c>
       <c r="I72" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
@@ -3580,7 +3580,7 @@
         </is>
       </c>
       <c r="I73" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
@@ -3621,7 +3621,7 @@
         </is>
       </c>
       <c r="I74" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="I75" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1">
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="I76" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
@@ -3744,7 +3744,7 @@
         </is>
       </c>
       <c r="I77" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
@@ -3785,7 +3785,7 @@
         </is>
       </c>
       <c r="I78" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
@@ -3826,7 +3826,7 @@
         </is>
       </c>
       <c r="I79" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="I80" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
@@ -3908,7 +3908,7 @@
         </is>
       </c>
       <c r="I81" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="I82" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="I83" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
@@ -4031,7 +4031,7 @@
         </is>
       </c>
       <c r="I84" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
@@ -4072,7 +4072,7 @@
         </is>
       </c>
       <c r="I85" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
@@ -4113,7 +4113,7 @@
         </is>
       </c>
       <c r="I86" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1">
@@ -4154,7 +4154,7 @@
         </is>
       </c>
       <c r="I87" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
@@ -4195,7 +4195,7 @@
         </is>
       </c>
       <c r="I88" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
@@ -4236,7 +4236,7 @@
         </is>
       </c>
       <c r="I89" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
@@ -4277,7 +4277,7 @@
         </is>
       </c>
       <c r="I90" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
@@ -4318,7 +4318,7 @@
         </is>
       </c>
       <c r="I91" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
@@ -4359,7 +4359,7 @@
         </is>
       </c>
       <c r="I92" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
@@ -4400,7 +4400,7 @@
         </is>
       </c>
       <c r="I93" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
@@ -4441,7 +4441,7 @@
         </is>
       </c>
       <c r="I94" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
@@ -4482,7 +4482,7 @@
         </is>
       </c>
       <c r="I95" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -4523,7 +4523,7 @@
         </is>
       </c>
       <c r="I96" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
@@ -4564,7 +4564,7 @@
         </is>
       </c>
       <c r="I97" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="I98" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
@@ -4646,7 +4646,7 @@
         </is>
       </c>
       <c r="I99" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="I100" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -4728,7 +4728,7 @@
         </is>
       </c>
       <c r="I101" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="I102" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1">
@@ -4810,7 +4810,7 @@
         </is>
       </c>
       <c r="I103" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="I104" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1">
@@ -4892,7 +4892,7 @@
         </is>
       </c>
       <c r="I105" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1">
@@ -4903,7 +4903,7 @@
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>14 B</t>
+          <t>14B</t>
         </is>
       </c>
       <c r="C106" s="9" t="inlineStr">
@@ -4933,7 +4933,7 @@
         </is>
       </c>
       <c r="I106" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
@@ -4974,7 +4974,7 @@
         </is>
       </c>
       <c r="I107" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1">
@@ -5015,7 +5015,7 @@
         </is>
       </c>
       <c r="I108" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1">
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="I109" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1">
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="I110" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" ht="15" customHeight="1">
@@ -5138,7 +5138,7 @@
         </is>
       </c>
       <c r="I111" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1">
@@ -5179,7 +5179,7 @@
         </is>
       </c>
       <c r="I112" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1">
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="I113" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" ht="15" customHeight="1">
@@ -5261,7 +5261,7 @@
         </is>
       </c>
       <c r="I114" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" ht="15" customHeight="1">
@@ -5302,7 +5302,7 @@
         </is>
       </c>
       <c r="I115" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" ht="15" customHeight="1">
@@ -5343,7 +5343,7 @@
         </is>
       </c>
       <c r="I116" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117" ht="15" customHeight="1">
@@ -5384,7 +5384,7 @@
         </is>
       </c>
       <c r="I117" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="118" ht="15" customHeight="1">
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="I118" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119" ht="15" customHeight="1">
@@ -5466,7 +5466,7 @@
         </is>
       </c>
       <c r="I119" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120" ht="15" customHeight="1">
@@ -5507,7 +5507,7 @@
         </is>
       </c>
       <c r="I120" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121" ht="15" customHeight="1">
@@ -5548,7 +5548,7 @@
         </is>
       </c>
       <c r="I121" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" ht="15" customHeight="1">
@@ -5589,7 +5589,7 @@
         </is>
       </c>
       <c r="I122" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123" ht="15" customHeight="1">
@@ -5630,7 +5630,7 @@
         </is>
       </c>
       <c r="I123" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" ht="15" customHeight="1">
@@ -5671,7 +5671,7 @@
         </is>
       </c>
       <c r="I124" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" ht="15" customHeight="1">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="I125" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" ht="15" customHeight="1">
@@ -5753,7 +5753,7 @@
         </is>
       </c>
       <c r="I126" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127" ht="15" customHeight="1">
@@ -5794,7 +5794,7 @@
         </is>
       </c>
       <c r="I127" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128" ht="15" customHeight="1">
@@ -5835,7 +5835,7 @@
         </is>
       </c>
       <c r="I128" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" ht="15" customHeight="1">
@@ -5876,7 +5876,7 @@
         </is>
       </c>
       <c r="I129" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" ht="15" customHeight="1">
@@ -5917,7 +5917,7 @@
         </is>
       </c>
       <c r="I130" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131" ht="15" customHeight="1">
@@ -5958,7 +5958,7 @@
         </is>
       </c>
       <c r="I131" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132" ht="15" customHeight="1">
@@ -5999,7 +5999,7 @@
         </is>
       </c>
       <c r="I132" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="133" ht="15" customHeight="1">
@@ -6040,7 +6040,7 @@
         </is>
       </c>
       <c r="I133" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134" ht="15" customHeight="1">
@@ -6081,7 +6081,7 @@
         </is>
       </c>
       <c r="I134" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135" ht="15" customHeight="1">
@@ -6122,7 +6122,7 @@
         </is>
       </c>
       <c r="I135" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136" ht="15" customHeight="1">
@@ -6163,7 +6163,7 @@
         </is>
       </c>
       <c r="I136" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137" ht="15" customHeight="1">
@@ -6204,7 +6204,7 @@
         </is>
       </c>
       <c r="I137" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138" ht="15" customHeight="1">
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="I138" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139" ht="15" customHeight="1">
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="I139" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140" ht="15" customHeight="1">
@@ -6321,7 +6321,7 @@
         </is>
       </c>
       <c r="I140" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141" ht="15" customHeight="1">
@@ -6362,7 +6362,7 @@
         </is>
       </c>
       <c r="I141" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142" ht="15" customHeight="1">
@@ -6403,7 +6403,7 @@
         </is>
       </c>
       <c r="I142" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143" ht="15" customHeight="1">
@@ -6444,7 +6444,7 @@
         </is>
       </c>
       <c r="I143" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144" ht="15" customHeight="1">
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="I144" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="145" ht="15" customHeight="1">
@@ -6526,7 +6526,7 @@
         </is>
       </c>
       <c r="I145" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146" ht="15" customHeight="1">
@@ -6567,7 +6567,7 @@
         </is>
       </c>
       <c r="I146" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147" ht="15" customHeight="1">
@@ -6608,7 +6608,7 @@
         </is>
       </c>
       <c r="I147" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148" ht="15" customHeight="1">
@@ -6649,7 +6649,7 @@
         </is>
       </c>
       <c r="I148" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" ht="15" customHeight="1">
@@ -6690,7 +6690,7 @@
         </is>
       </c>
       <c r="I149" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150" ht="15" customHeight="1">
@@ -6731,7 +6731,7 @@
         </is>
       </c>
       <c r="I150" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="151" ht="15" customHeight="1">
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="I151" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152" ht="15" customHeight="1">
@@ -6813,7 +6813,7 @@
         </is>
       </c>
       <c r="I152" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153" ht="15" customHeight="1">
@@ -6854,7 +6854,7 @@
         </is>
       </c>
       <c r="I153" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="154" ht="15" customHeight="1">
@@ -6895,7 +6895,7 @@
         </is>
       </c>
       <c r="I154" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155" ht="15" customHeight="1">
@@ -6936,7 +6936,7 @@
         </is>
       </c>
       <c r="I155" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156" ht="15" customHeight="1">
@@ -6977,7 +6977,7 @@
         </is>
       </c>
       <c r="I156" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157" ht="15" customHeight="1">
@@ -7018,7 +7018,7 @@
         </is>
       </c>
       <c r="I157" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158" ht="15" customHeight="1">
@@ -7059,7 +7059,7 @@
         </is>
       </c>
       <c r="I158" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159" ht="15" customHeight="1">
@@ -7100,7 +7100,7 @@
         </is>
       </c>
       <c r="I159" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160" ht="15" customHeight="1">
@@ -7141,7 +7141,7 @@
         </is>
       </c>
       <c r="I160" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161" ht="15" customHeight="1">
@@ -7182,7 +7182,7 @@
         </is>
       </c>
       <c r="I161" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162" ht="15" customHeight="1">
@@ -7223,7 +7223,7 @@
         </is>
       </c>
       <c r="I162" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163" ht="15" customHeight="1">
@@ -7264,7 +7264,7 @@
         </is>
       </c>
       <c r="I163" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="164" ht="15" customHeight="1">
@@ -7305,7 +7305,7 @@
         </is>
       </c>
       <c r="I164" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165" ht="15" customHeight="1">
@@ -7346,7 +7346,7 @@
         </is>
       </c>
       <c r="I165" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166" ht="15" customHeight="1">
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="I166" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167" ht="15" customHeight="1">
@@ -7428,7 +7428,7 @@
         </is>
       </c>
       <c r="I167" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168" ht="15" customHeight="1">
@@ -7469,7 +7469,7 @@
         </is>
       </c>
       <c r="I168" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169" ht="15" customHeight="1">
@@ -7510,7 +7510,7 @@
         </is>
       </c>
       <c r="I169" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170" ht="15" customHeight="1">
@@ -7551,7 +7551,7 @@
         </is>
       </c>
       <c r="I170" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171" ht="15" customHeight="1">
@@ -7592,7 +7592,7 @@
         </is>
       </c>
       <c r="I171" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172" ht="15" customHeight="1">
@@ -7633,7 +7633,7 @@
         </is>
       </c>
       <c r="I172" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173" ht="15" customHeight="1">
@@ -7674,7 +7674,7 @@
         </is>
       </c>
       <c r="I173" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174" ht="15" customHeight="1">
@@ -7715,7 +7715,7 @@
         </is>
       </c>
       <c r="I174" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175" ht="15" customHeight="1">
@@ -7756,7 +7756,7 @@
         </is>
       </c>
       <c r="I175" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176" ht="15" customHeight="1">
@@ -7797,7 +7797,7 @@
         </is>
       </c>
       <c r="I176" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177" ht="15" customHeight="1">
@@ -7838,7 +7838,7 @@
         </is>
       </c>
       <c r="I177" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178" ht="15" customHeight="1">
@@ -7879,7 +7879,7 @@
         </is>
       </c>
       <c r="I178" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="179" ht="15" customHeight="1">
@@ -7920,7 +7920,7 @@
         </is>
       </c>
       <c r="I179" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="180" ht="15" customHeight="1">
@@ -7961,7 +7961,7 @@
         </is>
       </c>
       <c r="I180" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="181" ht="15" customHeight="1">
@@ -8002,7 +8002,7 @@
         </is>
       </c>
       <c r="I181" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182" ht="15" customHeight="1">
@@ -8043,7 +8043,7 @@
         </is>
       </c>
       <c r="I182" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183" ht="15" customHeight="1">
@@ -8084,7 +8084,7 @@
         </is>
       </c>
       <c r="I183" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184" ht="15" customHeight="1">
@@ -8125,7 +8125,7 @@
         </is>
       </c>
       <c r="I184" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="185" ht="15" customHeight="1">
@@ -8166,7 +8166,7 @@
         </is>
       </c>
       <c r="I185" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186" ht="15" customHeight="1">
@@ -8207,7 +8207,7 @@
         </is>
       </c>
       <c r="I186" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="187" ht="15" customHeight="1">
@@ -8248,7 +8248,7 @@
         </is>
       </c>
       <c r="I187" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188" ht="15" customHeight="1">
@@ -8289,7 +8289,7 @@
         </is>
       </c>
       <c r="I188" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="189" ht="15" customHeight="1">
@@ -8330,7 +8330,7 @@
         </is>
       </c>
       <c r="I189" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190" ht="15" customHeight="1">
@@ -8371,7 +8371,7 @@
         </is>
       </c>
       <c r="I190" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="191" ht="15" customHeight="1">
@@ -8412,7 +8412,7 @@
         </is>
       </c>
       <c r="I191" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192" ht="15" customHeight="1">
@@ -8453,7 +8453,7 @@
         </is>
       </c>
       <c r="I192" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193" ht="15" customHeight="1">
@@ -8494,7 +8494,7 @@
         </is>
       </c>
       <c r="I193" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194" ht="15" customHeight="1">
@@ -8535,7 +8535,7 @@
         </is>
       </c>
       <c r="I194" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195" ht="15" customHeight="1">
@@ -8576,7 +8576,7 @@
         </is>
       </c>
       <c r="I195" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196" ht="15" customHeight="1">
@@ -8617,7 +8617,7 @@
         </is>
       </c>
       <c r="I196" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="197" ht="15" customHeight="1">
@@ -8658,7 +8658,7 @@
         </is>
       </c>
       <c r="I197" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198" ht="15" customHeight="1">
@@ -8699,7 +8699,7 @@
         </is>
       </c>
       <c r="I198" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="199" ht="15" customHeight="1">
@@ -8740,7 +8740,7 @@
         </is>
       </c>
       <c r="I199" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200" ht="15" customHeight="1">
@@ -8781,7 +8781,7 @@
         </is>
       </c>
       <c r="I200" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201" ht="15" customHeight="1">
@@ -8822,7 +8822,7 @@
         </is>
       </c>
       <c r="I201" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202" ht="15" customHeight="1">
@@ -8863,7 +8863,7 @@
         </is>
       </c>
       <c r="I202" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="203" ht="15" customHeight="1">
@@ -8904,7 +8904,7 @@
         </is>
       </c>
       <c r="I203" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="204" ht="15" customHeight="1">
@@ -8945,7 +8945,7 @@
         </is>
       </c>
       <c r="I204" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="205" ht="15" customHeight="1">
@@ -8986,7 +8986,7 @@
         </is>
       </c>
       <c r="I205" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206" ht="15" customHeight="1">
@@ -9027,7 +9027,7 @@
         </is>
       </c>
       <c r="I206" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207" ht="15" customHeight="1">
@@ -9068,7 +9068,7 @@
         </is>
       </c>
       <c r="I207" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208" ht="15" customHeight="1">
@@ -9109,7 +9109,7 @@
         </is>
       </c>
       <c r="I208" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209" ht="15" customHeight="1">
@@ -9150,7 +9150,7 @@
         </is>
       </c>
       <c r="I209" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210" ht="15" customHeight="1">
@@ -9191,7 +9191,7 @@
         </is>
       </c>
       <c r="I210" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="211" ht="15" customHeight="1">
@@ -9232,7 +9232,7 @@
         </is>
       </c>
       <c r="I211" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="212" ht="15" customHeight="1">
@@ -9273,7 +9273,7 @@
         </is>
       </c>
       <c r="I212" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="213" ht="15" customHeight="1">
@@ -9314,7 +9314,7 @@
         </is>
       </c>
       <c r="I213" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214" ht="15" customHeight="1">
@@ -9355,7 +9355,7 @@
         </is>
       </c>
       <c r="I214" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215" ht="15" customHeight="1">
@@ -9396,7 +9396,7 @@
         </is>
       </c>
       <c r="I215" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="216" ht="15" customHeight="1">
@@ -9437,7 +9437,7 @@
         </is>
       </c>
       <c r="I216" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217" ht="15" customHeight="1">
@@ -9478,7 +9478,7 @@
         </is>
       </c>
       <c r="I217" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="218" ht="15" customHeight="1">
@@ -9519,7 +9519,7 @@
         </is>
       </c>
       <c r="I218" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219" ht="15" customHeight="1">
@@ -9560,7 +9560,7 @@
         </is>
       </c>
       <c r="I219" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220" ht="15" customHeight="1">
@@ -9601,7 +9601,7 @@
         </is>
       </c>
       <c r="I220" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="221" ht="15" customHeight="1">
@@ -9642,7 +9642,7 @@
         </is>
       </c>
       <c r="I221" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="222" ht="15" customHeight="1">
@@ -9683,7 +9683,7 @@
         </is>
       </c>
       <c r="I222" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="223" ht="15" customHeight="1">
@@ -9724,7 +9724,7 @@
         </is>
       </c>
       <c r="I223" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="224" ht="15" customHeight="1">
@@ -9765,7 +9765,7 @@
         </is>
       </c>
       <c r="I224" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="225" ht="15" customHeight="1">
@@ -9806,7 +9806,7 @@
         </is>
       </c>
       <c r="I225" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226" ht="15" customHeight="1">
@@ -9847,7 +9847,7 @@
         </is>
       </c>
       <c r="I226" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="227" ht="15" customHeight="1">
@@ -9888,7 +9888,7 @@
         </is>
       </c>
       <c r="I227" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="228" ht="15" customHeight="1">
@@ -9929,7 +9929,7 @@
         </is>
       </c>
       <c r="I228" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="229" ht="15" customHeight="1">
@@ -9970,7 +9970,7 @@
         </is>
       </c>
       <c r="I229" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="230" ht="15" customHeight="1">
@@ -10011,7 +10011,7 @@
         </is>
       </c>
       <c r="I230" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231" ht="15" customHeight="1">
@@ -10052,7 +10052,7 @@
         </is>
       </c>
       <c r="I231" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="232" ht="15" customHeight="1">
@@ -10093,7 +10093,7 @@
         </is>
       </c>
       <c r="I232" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233" ht="15" customHeight="1">
@@ -10134,7 +10134,7 @@
         </is>
       </c>
       <c r="I233" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="234" ht="15" customHeight="1">
@@ -10175,7 +10175,7 @@
         </is>
       </c>
       <c r="I234" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="235" ht="15" customHeight="1">
@@ -10216,7 +10216,7 @@
         </is>
       </c>
       <c r="I235" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236" ht="15" customHeight="1">
@@ -10257,7 +10257,7 @@
         </is>
       </c>
       <c r="I236" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237" ht="15" customHeight="1">
@@ -10298,7 +10298,7 @@
         </is>
       </c>
       <c r="I237" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="238" ht="15" customHeight="1">
@@ -10339,7 +10339,7 @@
         </is>
       </c>
       <c r="I238" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239" ht="15" customHeight="1">
@@ -10380,7 +10380,7 @@
         </is>
       </c>
       <c r="I239" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="240" ht="15" customHeight="1">
@@ -10421,7 +10421,7 @@
         </is>
       </c>
       <c r="I240" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="241" ht="15" customHeight="1">
@@ -10462,7 +10462,7 @@
         </is>
       </c>
       <c r="I241" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="242" ht="15" customHeight="1">
@@ -10503,7 +10503,7 @@
         </is>
       </c>
       <c r="I242" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="243" ht="15" customHeight="1">
@@ -10544,7 +10544,7 @@
         </is>
       </c>
       <c r="I243" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="244" ht="15" customHeight="1">
@@ -10585,7 +10585,7 @@
         </is>
       </c>
       <c r="I244" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="245" ht="15" customHeight="1">
@@ -10626,7 +10626,7 @@
         </is>
       </c>
       <c r="I245" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="246" ht="15" customHeight="1">
@@ -10667,7 +10667,7 @@
         </is>
       </c>
       <c r="I246" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="247" ht="15" customHeight="1">
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="I247" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="248" ht="15" customHeight="1">
@@ -10749,7 +10749,7 @@
         </is>
       </c>
       <c r="I248" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="249" ht="15" customHeight="1">
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="I249" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="250" ht="15" customHeight="1">
@@ -10831,7 +10831,7 @@
         </is>
       </c>
       <c r="I250" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="251" ht="15" customHeight="1">
@@ -10872,7 +10872,7 @@
         </is>
       </c>
       <c r="I251" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="252" ht="15" customHeight="1">
@@ -10913,7 +10913,7 @@
         </is>
       </c>
       <c r="I252" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="253" ht="15" customHeight="1">
@@ -10954,7 +10954,7 @@
         </is>
       </c>
       <c r="I253" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="254" ht="15" customHeight="1">
@@ -10995,7 +10995,7 @@
         </is>
       </c>
       <c r="I254" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="255" ht="15" customHeight="1">
@@ -11036,7 +11036,7 @@
         </is>
       </c>
       <c r="I255" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="256" ht="15" customHeight="1">
@@ -11077,7 +11077,7 @@
         </is>
       </c>
       <c r="I256" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="257" ht="15" customHeight="1">
@@ -11118,7 +11118,7 @@
         </is>
       </c>
       <c r="I257" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="258" ht="15" customHeight="1">
@@ -11159,7 +11159,7 @@
         </is>
       </c>
       <c r="I258" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="259" ht="15" customHeight="1">
@@ -11200,7 +11200,7 @@
         </is>
       </c>
       <c r="I259" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="260" ht="15" customHeight="1">
@@ -11241,7 +11241,7 @@
         </is>
       </c>
       <c r="I260" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="261" ht="15" customHeight="1">
@@ -11282,7 +11282,7 @@
         </is>
       </c>
       <c r="I261" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="262" ht="15" customHeight="1">
@@ -11323,7 +11323,7 @@
         </is>
       </c>
       <c r="I262" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="263" ht="15" customHeight="1">
@@ -11364,7 +11364,7 @@
         </is>
       </c>
       <c r="I263" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="264" ht="15" customHeight="1">
@@ -11405,7 +11405,7 @@
         </is>
       </c>
       <c r="I264" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="265" ht="15" customHeight="1">
@@ -11446,7 +11446,7 @@
         </is>
       </c>
       <c r="I265" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="266" ht="15" customHeight="1">
@@ -11487,7 +11487,7 @@
         </is>
       </c>
       <c r="I266" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="267" ht="15" customHeight="1">
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="I267" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="268" ht="15" customHeight="1">
@@ -11569,7 +11569,7 @@
         </is>
       </c>
       <c r="I268" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="269" ht="15" customHeight="1">
@@ -11610,7 +11610,7 @@
         </is>
       </c>
       <c r="I269" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="270" ht="15" customHeight="1">
@@ -11651,7 +11651,7 @@
         </is>
       </c>
       <c r="I270" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="271" ht="15" customHeight="1">
@@ -11692,7 +11692,7 @@
         </is>
       </c>
       <c r="I271" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="272" ht="15" customHeight="1">
@@ -11733,7 +11733,7 @@
         </is>
       </c>
       <c r="I272" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="273" ht="15" customHeight="1">
@@ -11774,7 +11774,7 @@
         </is>
       </c>
       <c r="I273" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="274" ht="15" customHeight="1">
@@ -11815,7 +11815,7 @@
         </is>
       </c>
       <c r="I274" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="275" ht="15" customHeight="1">
@@ -11856,7 +11856,7 @@
         </is>
       </c>
       <c r="I275" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="276" ht="15" customHeight="1">
@@ -11897,7 +11897,7 @@
         </is>
       </c>
       <c r="I276" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="277" ht="15" customHeight="1">
@@ -11938,7 +11938,7 @@
         </is>
       </c>
       <c r="I277" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="278" ht="15" customHeight="1">
@@ -11979,7 +11979,7 @@
         </is>
       </c>
       <c r="I278" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="279" ht="15" customHeight="1">
@@ -12020,7 +12020,7 @@
         </is>
       </c>
       <c r="I279" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="280" ht="15" customHeight="1">
@@ -12061,7 +12061,7 @@
         </is>
       </c>
       <c r="I280" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="281" ht="15" customHeight="1">
@@ -12102,7 +12102,7 @@
         </is>
       </c>
       <c r="I281" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="282" ht="15" customHeight="1">
@@ -12143,7 +12143,7 @@
         </is>
       </c>
       <c r="I282" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283" ht="15" customHeight="1">
@@ -12184,7 +12184,7 @@
         </is>
       </c>
       <c r="I283" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="284" ht="15" customHeight="1">
@@ -12225,7 +12225,7 @@
         </is>
       </c>
       <c r="I284" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="285" ht="15" customHeight="1">
@@ -12266,7 +12266,7 @@
         </is>
       </c>
       <c r="I285" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="286" ht="15" customHeight="1">
@@ -12307,7 +12307,7 @@
         </is>
       </c>
       <c r="I286" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="287" ht="15" customHeight="1">
@@ -12348,7 +12348,7 @@
         </is>
       </c>
       <c r="I287" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="288" ht="15" customHeight="1">
@@ -12389,7 +12389,7 @@
         </is>
       </c>
       <c r="I288" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="289" ht="15" customHeight="1">
@@ -12430,7 +12430,7 @@
         </is>
       </c>
       <c r="I289" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="290" ht="15" customHeight="1">
@@ -12471,7 +12471,7 @@
         </is>
       </c>
       <c r="I290" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="291" ht="15" customHeight="1">
@@ -12512,7 +12512,7 @@
         </is>
       </c>
       <c r="I291" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="292" ht="15" customHeight="1">
@@ -12553,7 +12553,7 @@
         </is>
       </c>
       <c r="I292" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="293" ht="15" customHeight="1">
@@ -12594,7 +12594,7 @@
         </is>
       </c>
       <c r="I293" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="294" ht="15" customHeight="1">
@@ -12635,7 +12635,7 @@
         </is>
       </c>
       <c r="I294" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="295" ht="15" customHeight="1">
@@ -12676,7 +12676,7 @@
         </is>
       </c>
       <c r="I295" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="296" ht="15" customHeight="1">
@@ -12717,7 +12717,7 @@
         </is>
       </c>
       <c r="I296" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="297" ht="15" customHeight="1">
@@ -12758,7 +12758,7 @@
         </is>
       </c>
       <c r="I297" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="298" ht="15" customHeight="1">
@@ -12799,7 +12799,7 @@
         </is>
       </c>
       <c r="I298" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="299" ht="15" customHeight="1">
@@ -12840,7 +12840,7 @@
         </is>
       </c>
       <c r="I299" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="300" ht="15" customHeight="1">
@@ -12881,7 +12881,7 @@
         </is>
       </c>
       <c r="I300" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="301" ht="15" customHeight="1">
@@ -12922,7 +12922,7 @@
         </is>
       </c>
       <c r="I301" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="302" ht="15" customHeight="1">
@@ -12963,7 +12963,7 @@
         </is>
       </c>
       <c r="I302" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="303" ht="15" customHeight="1">
@@ -13004,7 +13004,7 @@
         </is>
       </c>
       <c r="I303" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="304" ht="15" customHeight="1">
@@ -13045,7 +13045,7 @@
         </is>
       </c>
       <c r="I304" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="305" ht="15" customHeight="1">
@@ -13086,7 +13086,7 @@
         </is>
       </c>
       <c r="I305" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="306" ht="15" customHeight="1">
@@ -13127,7 +13127,7 @@
         </is>
       </c>
       <c r="I306" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="307" ht="15" customHeight="1">
@@ -13168,7 +13168,7 @@
         </is>
       </c>
       <c r="I307" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="308" ht="15" customHeight="1">
@@ -13209,7 +13209,7 @@
         </is>
       </c>
       <c r="I308" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="309" ht="15" customHeight="1">
@@ -13250,7 +13250,7 @@
         </is>
       </c>
       <c r="I309" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="310" ht="15" customHeight="1">
@@ -13291,7 +13291,7 @@
         </is>
       </c>
       <c r="I310" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311" ht="15" customHeight="1">
@@ -13332,7 +13332,7 @@
         </is>
       </c>
       <c r="I311" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="312" ht="15" customHeight="1">
@@ -13373,7 +13373,7 @@
         </is>
       </c>
       <c r="I312" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="313" ht="15" customHeight="1">
@@ -13414,7 +13414,7 @@
         </is>
       </c>
       <c r="I313" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="314" ht="15" customHeight="1">
@@ -13455,7 +13455,7 @@
         </is>
       </c>
       <c r="I314" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="315" ht="15" customHeight="1">
@@ -13496,7 +13496,7 @@
         </is>
       </c>
       <c r="I315" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="316" ht="15" customHeight="1">
@@ -13537,7 +13537,7 @@
         </is>
       </c>
       <c r="I316" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="317" ht="15" customHeight="1">
@@ -13578,7 +13578,7 @@
         </is>
       </c>
       <c r="I317" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="318" ht="15" customHeight="1">
@@ -13619,7 +13619,7 @@
         </is>
       </c>
       <c r="I318" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="319" ht="15" customHeight="1">
@@ -13660,7 +13660,7 @@
         </is>
       </c>
       <c r="I319" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="320" ht="15" customHeight="1">
@@ -13701,7 +13701,7 @@
         </is>
       </c>
       <c r="I320" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="321" ht="15" customHeight="1">
@@ -13742,7 +13742,7 @@
         </is>
       </c>
       <c r="I321" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="322" ht="15" customHeight="1">
@@ -13783,7 +13783,7 @@
         </is>
       </c>
       <c r="I322" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="323" ht="15" customHeight="1">
@@ -13824,7 +13824,7 @@
         </is>
       </c>
       <c r="I323" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="324" ht="15" customHeight="1">
@@ -13865,7 +13865,7 @@
         </is>
       </c>
       <c r="I324" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="325" ht="15" customHeight="1">
@@ -13906,7 +13906,7 @@
         </is>
       </c>
       <c r="I325" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="326" ht="15" customHeight="1">
@@ -13947,7 +13947,7 @@
         </is>
       </c>
       <c r="I326" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="327" ht="15" customHeight="1">
@@ -13988,7 +13988,7 @@
         </is>
       </c>
       <c r="I327" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="328" ht="15" customHeight="1">
@@ -14029,7 +14029,7 @@
         </is>
       </c>
       <c r="I328" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="329" ht="15" customHeight="1">
@@ -14070,7 +14070,7 @@
         </is>
       </c>
       <c r="I329" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="330" ht="15" customHeight="1">
@@ -14111,7 +14111,7 @@
         </is>
       </c>
       <c r="I330" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="331" ht="15" customHeight="1">
@@ -14152,7 +14152,7 @@
         </is>
       </c>
       <c r="I331" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="332" ht="15" customHeight="1">
@@ -14193,7 +14193,7 @@
         </is>
       </c>
       <c r="I332" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="333" ht="15" customHeight="1">
@@ -14234,7 +14234,7 @@
         </is>
       </c>
       <c r="I333" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="334" ht="15" customHeight="1">
@@ -14275,7 +14275,7 @@
         </is>
       </c>
       <c r="I334" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="335" ht="15" customHeight="1">
@@ -14316,7 +14316,7 @@
         </is>
       </c>
       <c r="I335" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="336" ht="15" customHeight="1">
@@ -14357,7 +14357,7 @@
         </is>
       </c>
       <c r="I336" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="337" ht="15" customHeight="1">
@@ -14398,7 +14398,7 @@
         </is>
       </c>
       <c r="I337" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="338" ht="15" customHeight="1">
@@ -14439,7 +14439,7 @@
         </is>
       </c>
       <c r="I338" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="339" ht="15" customHeight="1">
@@ -14480,7 +14480,7 @@
         </is>
       </c>
       <c r="I339" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="340" ht="15" customHeight="1">
@@ -14521,7 +14521,7 @@
         </is>
       </c>
       <c r="I340" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="341" ht="15" customHeight="1">
@@ -14562,7 +14562,7 @@
         </is>
       </c>
       <c r="I341" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="342" ht="15" customHeight="1">
@@ -14603,7 +14603,7 @@
         </is>
       </c>
       <c r="I342" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="343" ht="15" customHeight="1">
@@ -14644,7 +14644,7 @@
         </is>
       </c>
       <c r="I343" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="344" ht="15" customHeight="1">
@@ -14685,7 +14685,7 @@
         </is>
       </c>
       <c r="I344" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="345" ht="15" customHeight="1">
@@ -14726,7 +14726,7 @@
         </is>
       </c>
       <c r="I345" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="346" ht="15" customHeight="1">
@@ -14767,7 +14767,7 @@
         </is>
       </c>
       <c r="I346" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="347" ht="15" customHeight="1">
@@ -14808,7 +14808,7 @@
         </is>
       </c>
       <c r="I347" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="348" ht="15" customHeight="1">
@@ -14849,7 +14849,7 @@
         </is>
       </c>
       <c r="I348" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="349" ht="15" customHeight="1">
@@ -14890,7 +14890,7 @@
         </is>
       </c>
       <c r="I349" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="350" ht="15" customHeight="1">
@@ -14931,7 +14931,7 @@
         </is>
       </c>
       <c r="I350" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="351" ht="15" customHeight="1">
@@ -14972,7 +14972,7 @@
         </is>
       </c>
       <c r="I351" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="352" ht="15" customHeight="1">
@@ -15013,7 +15013,7 @@
         </is>
       </c>
       <c r="I352" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="353" ht="15" customHeight="1">
@@ -15054,7 +15054,7 @@
         </is>
       </c>
       <c r="I353" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="354" ht="15" customHeight="1">
@@ -15095,7 +15095,7 @@
         </is>
       </c>
       <c r="I354" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="355" ht="15" customHeight="1">
@@ -15136,7 +15136,7 @@
         </is>
       </c>
       <c r="I355" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="356" ht="15" customHeight="1">
@@ -15177,7 +15177,7 @@
         </is>
       </c>
       <c r="I356" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="357" ht="15" customHeight="1">
@@ -15218,7 +15218,7 @@
         </is>
       </c>
       <c r="I357" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="358" ht="15" customHeight="1">
@@ -15259,7 +15259,7 @@
         </is>
       </c>
       <c r="I358" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="359" ht="15" customHeight="1">
@@ -15300,7 +15300,7 @@
         </is>
       </c>
       <c r="I359" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="360" ht="15" customHeight="1">
@@ -15341,7 +15341,7 @@
         </is>
       </c>
       <c r="I360" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="361" ht="15" customHeight="1">
@@ -15382,7 +15382,7 @@
         </is>
       </c>
       <c r="I361" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="362" ht="15" customHeight="1">
@@ -15423,7 +15423,7 @@
         </is>
       </c>
       <c r="I362" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="363" ht="15" customHeight="1">
@@ -15464,7 +15464,7 @@
         </is>
       </c>
       <c r="I363" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="364" ht="15" customHeight="1">
@@ -15505,7 +15505,7 @@
         </is>
       </c>
       <c r="I364" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="365" ht="15" customHeight="1">
@@ -15546,7 +15546,7 @@
         </is>
       </c>
       <c r="I365" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="366" ht="15" customHeight="1">
@@ -15587,7 +15587,7 @@
         </is>
       </c>
       <c r="I366" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="367" ht="15" customHeight="1">
@@ -15628,7 +15628,7 @@
         </is>
       </c>
       <c r="I367" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="368" ht="15" customHeight="1">
@@ -15669,7 +15669,7 @@
         </is>
       </c>
       <c r="I368" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="369" ht="15" customHeight="1">
@@ -15710,7 +15710,7 @@
         </is>
       </c>
       <c r="I369" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="370" ht="15" customHeight="1">
@@ -15751,7 +15751,7 @@
         </is>
       </c>
       <c r="I370" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="371" ht="15" customHeight="1">
@@ -15792,7 +15792,7 @@
         </is>
       </c>
       <c r="I371" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="372" ht="15" customHeight="1">
@@ -15833,7 +15833,7 @@
         </is>
       </c>
       <c r="I372" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="373" ht="15" customHeight="1">
@@ -15874,7 +15874,7 @@
         </is>
       </c>
       <c r="I373" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="374" ht="15" customHeight="1">
@@ -15915,7 +15915,7 @@
         </is>
       </c>
       <c r="I374" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="375" ht="15" customHeight="1">
@@ -15956,7 +15956,7 @@
         </is>
       </c>
       <c r="I375" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="376" ht="15" customHeight="1">
@@ -15997,7 +15997,7 @@
         </is>
       </c>
       <c r="I376" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="377" ht="15" customHeight="1">
@@ -16038,7 +16038,7 @@
         </is>
       </c>
       <c r="I377" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="378" ht="15" customHeight="1">
@@ -16079,7 +16079,7 @@
         </is>
       </c>
       <c r="I378" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="379" ht="15" customHeight="1">
@@ -16120,7 +16120,7 @@
         </is>
       </c>
       <c r="I379" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="380" ht="15" customHeight="1">
@@ -16161,7 +16161,7 @@
         </is>
       </c>
       <c r="I380" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="381" ht="15" customHeight="1">
@@ -16202,7 +16202,7 @@
         </is>
       </c>
       <c r="I381" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="382" ht="15" customHeight="1">
@@ -16243,7 +16243,7 @@
         </is>
       </c>
       <c r="I382" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="383" ht="15" customHeight="1">
@@ -16284,7 +16284,7 @@
         </is>
       </c>
       <c r="I383" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="384" ht="15" customHeight="1">
@@ -16325,7 +16325,7 @@
         </is>
       </c>
       <c r="I384" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="385" ht="15" customHeight="1">
@@ -16366,7 +16366,7 @@
         </is>
       </c>
       <c r="I385" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="386" ht="15" customHeight="1">
@@ -16407,7 +16407,7 @@
         </is>
       </c>
       <c r="I386" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="387" ht="15" customHeight="1">
@@ -16448,7 +16448,7 @@
         </is>
       </c>
       <c r="I387" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="388" ht="15" customHeight="1">
@@ -16489,7 +16489,7 @@
         </is>
       </c>
       <c r="I388" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="389" ht="15" customHeight="1">
@@ -16530,7 +16530,7 @@
         </is>
       </c>
       <c r="I389" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="390" ht="15" customHeight="1">
@@ -16571,7 +16571,7 @@
         </is>
       </c>
       <c r="I390" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="391" ht="15" customHeight="1">
@@ -16612,7 +16612,7 @@
         </is>
       </c>
       <c r="I391" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="392" ht="15" customHeight="1">
@@ -16653,7 +16653,7 @@
         </is>
       </c>
       <c r="I392" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="393" ht="15" customHeight="1">
@@ -16694,7 +16694,7 @@
         </is>
       </c>
       <c r="I393" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="394" ht="15" customHeight="1">
@@ -16735,7 +16735,7 @@
         </is>
       </c>
       <c r="I394" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="395" ht="15" customHeight="1">
@@ -16776,7 +16776,7 @@
         </is>
       </c>
       <c r="I395" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="396" ht="15" customHeight="1">
@@ -16817,7 +16817,7 @@
         </is>
       </c>
       <c r="I396" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="397" ht="15" customHeight="1">
@@ -16858,7 +16858,7 @@
         </is>
       </c>
       <c r="I397" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="398" ht="15" customHeight="1">
@@ -16899,7 +16899,7 @@
         </is>
       </c>
       <c r="I398" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="399" ht="15" customHeight="1">
@@ -16940,7 +16940,7 @@
         </is>
       </c>
       <c r="I399" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="400" ht="15" customHeight="1">
@@ -16981,7 +16981,7 @@
         </is>
       </c>
       <c r="I400" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="401" ht="15" customHeight="1">
@@ -17022,7 +17022,7 @@
         </is>
       </c>
       <c r="I401" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="402" ht="15" customHeight="1">
@@ -17063,7 +17063,7 @@
         </is>
       </c>
       <c r="I402" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="403" ht="15" customHeight="1">
@@ -17104,7 +17104,7 @@
         </is>
       </c>
       <c r="I403" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="404" ht="15" customHeight="1">
@@ -17145,7 +17145,7 @@
         </is>
       </c>
       <c r="I404" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="405" ht="15" customHeight="1">
@@ -17186,7 +17186,7 @@
         </is>
       </c>
       <c r="I405" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="406" ht="15" customHeight="1">
@@ -17227,7 +17227,7 @@
         </is>
       </c>
       <c r="I406" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="407" ht="15" customHeight="1">
@@ -17268,7 +17268,7 @@
         </is>
       </c>
       <c r="I407" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="408" ht="15" customHeight="1">
@@ -17309,7 +17309,7 @@
         </is>
       </c>
       <c r="I408" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="409" ht="15" customHeight="1">
@@ -17350,7 +17350,7 @@
         </is>
       </c>
       <c r="I409" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="410" ht="15" customHeight="1">
@@ -17391,7 +17391,7 @@
         </is>
       </c>
       <c r="I410" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="411" ht="15" customHeight="1">
@@ -17432,7 +17432,7 @@
         </is>
       </c>
       <c r="I411" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="412" ht="15" customHeight="1">
@@ -17471,7 +17471,7 @@
         </is>
       </c>
       <c r="I412" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="413" ht="15" customHeight="1">
@@ -17512,7 +17512,7 @@
         </is>
       </c>
       <c r="I413" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="414" ht="15" customHeight="1">
@@ -17553,7 +17553,7 @@
         </is>
       </c>
       <c r="I414" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="415" ht="15" customHeight="1">
@@ -17594,7 +17594,7 @@
         </is>
       </c>
       <c r="I415" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="416" ht="15" customHeight="1">
@@ -17635,7 +17635,7 @@
         </is>
       </c>
       <c r="I416" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="417" ht="15" customHeight="1">
@@ -17676,7 +17676,7 @@
         </is>
       </c>
       <c r="I417" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="418" ht="15" customHeight="1">
@@ -17717,7 +17717,7 @@
         </is>
       </c>
       <c r="I418" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="419" ht="15" customHeight="1">
@@ -17758,7 +17758,7 @@
         </is>
       </c>
       <c r="I419" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="420" ht="15" customHeight="1">
@@ -17799,7 +17799,7 @@
         </is>
       </c>
       <c r="I420" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="421" ht="15" customHeight="1">
@@ -17840,7 +17840,7 @@
         </is>
       </c>
       <c r="I421" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="422" ht="15" customHeight="1">
@@ -17881,7 +17881,7 @@
         </is>
       </c>
       <c r="I422" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="423" ht="15" customHeight="1">
@@ -17922,7 +17922,7 @@
         </is>
       </c>
       <c r="I423" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="424" ht="15" customHeight="1">
@@ -17963,7 +17963,7 @@
         </is>
       </c>
       <c r="I424" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="425" ht="15" customHeight="1">
@@ -18004,7 +18004,7 @@
         </is>
       </c>
       <c r="I425" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="426" ht="15" customHeight="1">
@@ -18045,7 +18045,7 @@
         </is>
       </c>
       <c r="I426" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="427" ht="15" customHeight="1">
@@ -18086,7 +18086,7 @@
         </is>
       </c>
       <c r="I427" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="428" ht="15" customHeight="1">
@@ -18127,7 +18127,7 @@
         </is>
       </c>
       <c r="I428" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="429" ht="15" customHeight="1">
@@ -18168,7 +18168,7 @@
         </is>
       </c>
       <c r="I429" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="430" ht="15" customHeight="1">
@@ -18209,7 +18209,7 @@
         </is>
       </c>
       <c r="I430" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="431" ht="15" customHeight="1">
@@ -18250,7 +18250,7 @@
         </is>
       </c>
       <c r="I431" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="432" ht="15" customHeight="1">
@@ -18291,7 +18291,7 @@
         </is>
       </c>
       <c r="I432" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="433" ht="15" customHeight="1">
@@ -18332,7 +18332,7 @@
         </is>
       </c>
       <c r="I433" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="434" ht="15" customHeight="1">
@@ -18373,7 +18373,7 @@
         </is>
       </c>
       <c r="I434" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="435" ht="15" customHeight="1">
@@ -18414,7 +18414,7 @@
         </is>
       </c>
       <c r="I435" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="436" ht="15" customHeight="1">
@@ -18455,7 +18455,7 @@
         </is>
       </c>
       <c r="I436" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="437" ht="15" customHeight="1">
@@ -18496,7 +18496,7 @@
         </is>
       </c>
       <c r="I437" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="438" ht="15" customHeight="1">
@@ -18537,7 +18537,7 @@
         </is>
       </c>
       <c r="I438" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="439" ht="15" customHeight="1">
@@ -18578,7 +18578,7 @@
         </is>
       </c>
       <c r="I439" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="440" ht="15" customHeight="1">
@@ -18619,7 +18619,7 @@
         </is>
       </c>
       <c r="I440" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="441" ht="15" customHeight="1">
@@ -18660,7 +18660,7 @@
         </is>
       </c>
       <c r="I441" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="442" ht="15" customHeight="1">
@@ -18701,7 +18701,7 @@
         </is>
       </c>
       <c r="I442" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="443" ht="15" customHeight="1">
@@ -18742,7 +18742,7 @@
         </is>
       </c>
       <c r="I443" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="444" ht="15" customHeight="1">
@@ -18783,7 +18783,7 @@
         </is>
       </c>
       <c r="I444" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="445" ht="15" customHeight="1">
@@ -18824,7 +18824,7 @@
         </is>
       </c>
       <c r="I445" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="446" ht="15" customHeight="1">
@@ -18865,7 +18865,7 @@
         </is>
       </c>
       <c r="I446" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="447" ht="15" customHeight="1">
@@ -18906,7 +18906,7 @@
         </is>
       </c>
       <c r="I447" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="448" ht="15" customHeight="1">
@@ -18947,7 +18947,7 @@
         </is>
       </c>
       <c r="I448" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="449" ht="15" customHeight="1">
@@ -18988,7 +18988,7 @@
         </is>
       </c>
       <c r="I449" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="450" ht="15" customHeight="1">
@@ -19029,7 +19029,7 @@
         </is>
       </c>
       <c r="I450" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="451" ht="15" customHeight="1">
@@ -19070,7 +19070,7 @@
         </is>
       </c>
       <c r="I451" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="452" ht="15" customHeight="1">
@@ -19111,7 +19111,7 @@
         </is>
       </c>
       <c r="I452" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="453" ht="15" customHeight="1">
@@ -19152,7 +19152,7 @@
         </is>
       </c>
       <c r="I453" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="454" ht="15" customHeight="1">
@@ -19193,7 +19193,7 @@
         </is>
       </c>
       <c r="I454" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="455" ht="15" customHeight="1">
@@ -19234,7 +19234,7 @@
         </is>
       </c>
       <c r="I455" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="456" ht="15" customHeight="1">
@@ -19275,7 +19275,7 @@
         </is>
       </c>
       <c r="I456" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="457" ht="15" customHeight="1">
@@ -19316,7 +19316,7 @@
         </is>
       </c>
       <c r="I457" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="458" ht="15" customHeight="1">
@@ -19357,7 +19357,7 @@
         </is>
       </c>
       <c r="I458" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="459" ht="15" customHeight="1">
@@ -19398,7 +19398,7 @@
         </is>
       </c>
       <c r="I459" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="460" ht="15" customHeight="1">
@@ -19439,7 +19439,7 @@
         </is>
       </c>
       <c r="I460" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="461" ht="15" customHeight="1">
@@ -19480,7 +19480,7 @@
         </is>
       </c>
       <c r="I461" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="462" ht="15" customHeight="1">
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="I462" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="463" ht="15" customHeight="1">
@@ -19562,7 +19562,7 @@
         </is>
       </c>
       <c r="I463" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="464" ht="15" customHeight="1">
@@ -19603,7 +19603,7 @@
         </is>
       </c>
       <c r="I464" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="465" ht="15" customHeight="1">
@@ -19644,7 +19644,7 @@
         </is>
       </c>
       <c r="I465" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="466" ht="15" customHeight="1">
@@ -19685,7 +19685,7 @@
         </is>
       </c>
       <c r="I466" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="467" ht="15" customHeight="1">
@@ -19726,7 +19726,7 @@
         </is>
       </c>
       <c r="I467" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="468" ht="15" customHeight="1">
@@ -19767,7 +19767,7 @@
         </is>
       </c>
       <c r="I468" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="469" ht="15" customHeight="1">
@@ -19808,7 +19808,7 @@
         </is>
       </c>
       <c r="I469" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="470" ht="15" customHeight="1">
@@ -19849,7 +19849,7 @@
         </is>
       </c>
       <c r="I470" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="471" ht="15" customHeight="1">
@@ -19890,7 +19890,7 @@
         </is>
       </c>
       <c r="I471" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="472" ht="15" customHeight="1">
@@ -19931,7 +19931,7 @@
         </is>
       </c>
       <c r="I472" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="473" ht="15" customHeight="1">
@@ -19972,7 +19972,7 @@
         </is>
       </c>
       <c r="I473" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="474" ht="15" customHeight="1">
@@ -20013,7 +20013,7 @@
         </is>
       </c>
       <c r="I474" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="475" ht="15" customHeight="1">
@@ -20054,7 +20054,7 @@
         </is>
       </c>
       <c r="I475" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="476" ht="15" customHeight="1">
@@ -20095,7 +20095,7 @@
         </is>
       </c>
       <c r="I476" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="477" ht="15" customHeight="1">
@@ -20136,7 +20136,7 @@
         </is>
       </c>
       <c r="I477" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="478" ht="15" customHeight="1">
@@ -20177,7 +20177,7 @@
         </is>
       </c>
       <c r="I478" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="479" ht="15" customHeight="1">
@@ -20218,7 +20218,7 @@
         </is>
       </c>
       <c r="I479" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="480" ht="15" customHeight="1">
@@ -20259,7 +20259,7 @@
         </is>
       </c>
       <c r="I480" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="481" ht="15" customHeight="1">
@@ -20300,7 +20300,7 @@
         </is>
       </c>
       <c r="I481" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="482" ht="15" customHeight="1">
@@ -20341,7 +20341,7 @@
         </is>
       </c>
       <c r="I482" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="483" ht="15" customHeight="1">
@@ -20382,7 +20382,7 @@
         </is>
       </c>
       <c r="I483" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="484" ht="15" customHeight="1">
@@ -20423,7 +20423,7 @@
         </is>
       </c>
       <c r="I484" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="485" ht="15" customHeight="1">
@@ -20464,7 +20464,7 @@
         </is>
       </c>
       <c r="I485" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="486" ht="15" customHeight="1">
@@ -20505,7 +20505,7 @@
         </is>
       </c>
       <c r="I486" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="487" ht="15" customHeight="1">
@@ -20546,7 +20546,7 @@
         </is>
       </c>
       <c r="I487" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="488" ht="15" customHeight="1">
@@ -20587,7 +20587,7 @@
         </is>
       </c>
       <c r="I488" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="489" ht="15" customHeight="1">
@@ -20628,7 +20628,7 @@
         </is>
       </c>
       <c r="I489" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="490" ht="15" customHeight="1">
@@ -20669,7 +20669,7 @@
         </is>
       </c>
       <c r="I490" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="491" ht="15" customHeight="1">
@@ -20710,7 +20710,7 @@
         </is>
       </c>
       <c r="I491" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="492" ht="15" customHeight="1">
@@ -20751,7 +20751,7 @@
         </is>
       </c>
       <c r="I492" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="493" ht="15" customHeight="1">
@@ -20792,7 +20792,7 @@
         </is>
       </c>
       <c r="I493" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="494" ht="15" customHeight="1">
@@ -20833,7 +20833,7 @@
         </is>
       </c>
       <c r="I494" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="495" ht="15" customHeight="1">
@@ -20874,7 +20874,7 @@
         </is>
       </c>
       <c r="I495" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="496" ht="15" customHeight="1">
@@ -20915,7 +20915,7 @@
         </is>
       </c>
       <c r="I496" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="497" ht="15" customHeight="1">
@@ -20956,7 +20956,7 @@
         </is>
       </c>
       <c r="I497" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="498" ht="15" customHeight="1">
@@ -20997,7 +20997,7 @@
         </is>
       </c>
       <c r="I498" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="499" ht="15" customHeight="1">
@@ -21038,7 +21038,7 @@
         </is>
       </c>
       <c r="I499" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="500" ht="15" customHeight="1">
@@ -21079,7 +21079,7 @@
         </is>
       </c>
       <c r="I500" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="501" ht="15" customHeight="1">
@@ -21120,7 +21120,7 @@
         </is>
       </c>
       <c r="I501" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="502" ht="15" customHeight="1">
@@ -21161,7 +21161,7 @@
         </is>
       </c>
       <c r="I502" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="503" ht="15" customHeight="1">
@@ -21202,7 +21202,7 @@
         </is>
       </c>
       <c r="I503" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="504" ht="15" customHeight="1">
@@ -21243,7 +21243,7 @@
         </is>
       </c>
       <c r="I504" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="505" ht="15" customHeight="1">
@@ -21284,7 +21284,7 @@
         </is>
       </c>
       <c r="I505" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="506" ht="15" customHeight="1">
@@ -21325,7 +21325,7 @@
         </is>
       </c>
       <c r="I506" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="507" ht="15" customHeight="1">
@@ -21364,7 +21364,7 @@
         </is>
       </c>
       <c r="I507" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="508" ht="15" customHeight="1">
@@ -21403,7 +21403,7 @@
         </is>
       </c>
       <c r="I508" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="509" ht="15" customHeight="1">
@@ -21444,7 +21444,7 @@
         </is>
       </c>
       <c r="I509" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="510" ht="15" customHeight="1">
@@ -21485,7 +21485,7 @@
         </is>
       </c>
       <c r="I510" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="511" ht="15" customHeight="1">
@@ -21526,7 +21526,7 @@
         </is>
       </c>
       <c r="I511" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>